<commit_message>
chore(holomap): synchronise le gabarit Excel + re-bake l'instantané
Carte Holo/carte_holomap.xlsx édité par Rhend, instantané re-baké
(tools/bake_holomap.gd) pour rester à jour — TestHoloXlsx (CI) l'exige.

Vérifié : TestHoloXlsx 0 échec (aller-retour, fallback build, instantané
à jour).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011uxYWWW692nqmByu8Cuzfw
</commit_message>
<xml_diff>
--- a/Carte Holo/carte_holomap.xlsx
+++ b/Carte Holo/carte_holomap.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projets\IdleEvolution\Carte Holo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\b.consol\Downloads\Divers\ecole\Dossier UE9\Reliquary\Carte Holo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ACAEED3-5A76-4511-BF7D-C8D8030C8471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B15A1B-B4EF-4C9D-BA1E-D70D1CACF421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Paramètres" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="200">
   <si>
     <t>Paramètres globaux — HoloMap</t>
   </si>
@@ -290,12 +290,6 @@
     <t>Note</t>
   </si>
   <si>
-    <t>biome_marais</t>
-  </si>
-  <si>
-    <t>(exemple — à remplacer)</t>
-  </si>
-  <si>
     <t>Remplir avec les ids réels des .tres de lieux. Cette liste est un aide-mémoire des ids valides à écrire dans la grille ; la source d'autorité reste les .tres.</t>
   </si>
   <si>
@@ -479,24 +473,15 @@
     <t>9c</t>
   </si>
   <si>
-    <t>biome_montagne</t>
-  </si>
-  <si>
     <t>24g</t>
   </si>
   <si>
     <t>10d</t>
   </si>
   <si>
-    <t>biome_marecage</t>
-  </si>
-  <si>
     <t>12g</t>
   </si>
   <si>
-    <t>biome_foret</t>
-  </si>
-  <si>
     <t>12p</t>
   </si>
   <si>
@@ -644,13 +629,16 @@
     <t>Bâtiment industriel à l'abandon, métal corrodé (motif libre).</t>
   </si>
   <si>
-    <t>biome_colline</t>
-  </si>
-  <si>
-    <t>biome_ville_fantome</t>
-  </si>
-  <si>
-    <t>biome_cimetiere</t>
+    <t>biome_usine</t>
+  </si>
+  <si>
+    <t>Usines</t>
+  </si>
+  <si>
+    <t>biome_usines</t>
+  </si>
+  <si>
+    <t>C'est l'usine</t>
   </si>
 </sst>
 </file>
@@ -1947,7 +1935,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="210">
+  <cellXfs count="212">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2159,26 +2147,6 @@
     <xf numFmtId="0" fontId="0" fillId="30" borderId="41" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="30" borderId="42" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="30" borderId="43" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -2188,6 +2156,32 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2504,11 +2498,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="195" t="s">
+      <c r="A1" s="202" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="196"/>
-      <c r="C1" s="196"/>
+      <c r="B1" s="201"/>
+      <c r="C1" s="201"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -2566,11 +2560,11 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="197" t="s">
+      <c r="A9" s="208" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="196"/>
-      <c r="C9" s="196"/>
+      <c r="B9" s="201"/>
+      <c r="C9" s="201"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3213,7 +3207,7 @@
       <c r="AR8" s="36"/>
       <c r="AS8" s="41"/>
       <c r="AT8" s="22" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="AU8" s="22"/>
       <c r="AV8" s="42"/>
@@ -3504,9 +3498,7 @@
       <c r="F13" s="7"/>
       <c r="G13" s="36"/>
       <c r="H13" s="51"/>
-      <c r="I13" s="52" t="s">
-        <v>201</v>
-      </c>
+      <c r="I13" s="52"/>
       <c r="J13" s="52"/>
       <c r="K13" s="52"/>
       <c r="L13" s="52"/>
@@ -3679,9 +3671,7 @@
       <c r="AW15" s="57"/>
       <c r="AX15" s="58"/>
       <c r="AY15" s="58"/>
-      <c r="AZ15" s="58" t="s">
-        <v>203</v>
-      </c>
+      <c r="AZ15" s="58"/>
       <c r="BA15" s="58"/>
       <c r="BB15" s="58"/>
       <c r="BC15" s="59"/>
@@ -3862,7 +3852,7 @@
       <c r="AI18" s="69"/>
       <c r="AJ18" s="70"/>
       <c r="AK18" s="70" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="AL18" s="70"/>
       <c r="AM18" s="70"/>
@@ -4049,7 +4039,7 @@
       <c r="Y21" s="82"/>
       <c r="Z21" s="83"/>
       <c r="AA21" s="83" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="AB21" s="83"/>
       <c r="AC21" s="84"/>
@@ -4729,7 +4719,7 @@
       <c r="AC31" s="109"/>
       <c r="AD31" s="70"/>
       <c r="AE31" s="70" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="AF31" s="70"/>
       <c r="AG31" s="110"/>
@@ -4742,9 +4732,7 @@
       <c r="AN31" s="62"/>
       <c r="AO31" s="111"/>
       <c r="AP31" s="112"/>
-      <c r="AQ31" s="112" t="s">
-        <v>149</v>
-      </c>
+      <c r="AQ31" s="112"/>
       <c r="AR31" s="112"/>
       <c r="AS31" s="112"/>
       <c r="AT31" s="112"/>
@@ -4796,9 +4784,7 @@
       <c r="AA32" s="10"/>
       <c r="AB32" s="62"/>
       <c r="AC32" s="109"/>
-      <c r="AD32" s="70" t="s">
-        <v>146</v>
-      </c>
+      <c r="AD32" s="70"/>
       <c r="AE32" s="70"/>
       <c r="AF32" s="70"/>
       <c r="AG32" s="110"/>
@@ -5126,7 +5112,7 @@
       <c r="AD37" s="70"/>
       <c r="AE37" s="70"/>
       <c r="AF37" s="70" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="AG37" s="70"/>
       <c r="AH37" s="71"/>
@@ -5273,9 +5259,7 @@
       <c r="AS39" s="123"/>
       <c r="AT39" s="124"/>
       <c r="AU39" s="124"/>
-      <c r="AV39" s="124" t="s">
-        <v>151</v>
-      </c>
+      <c r="AV39" s="124"/>
       <c r="AW39" s="124"/>
       <c r="AX39" s="124"/>
       <c r="AY39" s="124"/>
@@ -5886,9 +5870,7 @@
       <c r="F49" s="7"/>
       <c r="G49" s="36"/>
       <c r="H49" s="133"/>
-      <c r="I49" s="134" t="s">
-        <v>202</v>
-      </c>
+      <c r="I49" s="134"/>
       <c r="J49" s="134"/>
       <c r="K49" s="135"/>
       <c r="L49" s="78"/>
@@ -6155,7 +6137,9 @@
       <c r="M53" s="7"/>
       <c r="N53" s="36"/>
       <c r="O53" s="136"/>
-      <c r="P53" s="137"/>
+      <c r="P53" s="137" t="s">
+        <v>196</v>
+      </c>
       <c r="Q53" s="137"/>
       <c r="R53" s="137"/>
       <c r="S53" s="137"/>
@@ -6729,831 +6713,835 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D99"/>
+  <dimension ref="B1:E99"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="60" customWidth="1"/>
+    <col min="1" max="1" width="1.85546875" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="195" t="s">
+    <row r="1" spans="2:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B1" s="202" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="196"/>
-      <c r="C1" s="196"/>
-      <c r="D1" s="196"/>
-    </row>
-    <row r="3" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="201" t="s">
+      <c r="C1" s="201"/>
+      <c r="D1" s="201"/>
+      <c r="E1" s="201"/>
+    </row>
+    <row r="3" spans="2:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="204" t="s">
         <v>43</v>
       </c>
-      <c r="B3" s="196"/>
-      <c r="C3" s="196"/>
-      <c r="D3" s="196"/>
-    </row>
-    <row r="4" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="196"/>
-      <c r="B4" s="196"/>
-      <c r="C4" s="196"/>
-      <c r="D4" s="196"/>
-    </row>
-    <row r="5" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="196"/>
-      <c r="B5" s="196"/>
-      <c r="C5" s="196"/>
-      <c r="D5" s="196"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="C3" s="201"/>
+      <c r="D3" s="201"/>
+      <c r="E3" s="201"/>
+    </row>
+    <row r="4" spans="2:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="201"/>
+      <c r="C4" s="201"/>
+      <c r="D4" s="201"/>
+      <c r="E4" s="201"/>
+    </row>
+    <row r="5" spans="2:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="201"/>
+      <c r="C5" s="201"/>
+      <c r="D5" s="201"/>
+      <c r="E5" s="201"/>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="202" t="s">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="205" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="196"/>
-      <c r="C8" s="196"/>
-      <c r="D8" s="196"/>
-    </row>
-    <row r="9" spans="1:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="A9" s="20"/>
-      <c r="B9" s="2" t="s">
+      <c r="C8" s="201"/>
+      <c r="D8" s="201"/>
+      <c r="E8" s="201"/>
+    </row>
+    <row r="9" spans="2:5" ht="24" x14ac:dyDescent="0.25">
+      <c r="B9" s="20"/>
+      <c r="C9" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="D9" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="10"/>
-      <c r="B10" s="2" t="s">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="10"/>
+      <c r="C10" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="D10" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="22"/>
-      <c r="B11" s="2" t="s">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B11" s="22"/>
+      <c r="C11" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="D11" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="E11" s="4" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="23"/>
-      <c r="B12" s="2" t="s">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B12" s="23"/>
+      <c r="C12" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="D12" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="A13" s="24"/>
-      <c r="B13" s="2" t="s">
+    <row r="13" spans="2:5" ht="24" x14ac:dyDescent="0.25">
+      <c r="B13" s="24"/>
+      <c r="C13" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="D13" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="A14" s="25"/>
-      <c r="B14" s="2" t="s">
+    <row r="14" spans="2:5" ht="24" x14ac:dyDescent="0.25">
+      <c r="B14" s="25"/>
+      <c r="C14" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="D14" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="209"/>
-      <c r="B15" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="C15" s="21" t="s">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B15" s="199"/>
+      <c r="C15" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D15" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="208"/>
-      <c r="B16" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="C16" s="21" t="s">
+      <c r="E15" s="4" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B16" s="198"/>
+      <c r="C16" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="D16" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="E16" s="4" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="36" x14ac:dyDescent="0.25">
+      <c r="B17" s="174"/>
+      <c r="C17" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="24" x14ac:dyDescent="0.25">
+      <c r="B18" s="175"/>
+      <c r="C18" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="D18" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="24" x14ac:dyDescent="0.25">
+      <c r="B19" s="176"/>
+      <c r="C19" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D19" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="24" x14ac:dyDescent="0.25">
+      <c r="B20" s="26"/>
+      <c r="C20" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D20" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="24" x14ac:dyDescent="0.25">
+      <c r="B21" s="27"/>
+      <c r="C21" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" ht="36" x14ac:dyDescent="0.25">
+      <c r="B22" s="162"/>
+      <c r="C22" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" ht="36" x14ac:dyDescent="0.25">
+      <c r="B23" s="28"/>
+      <c r="C23" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" ht="24" x14ac:dyDescent="0.25">
+      <c r="B24" s="29"/>
+      <c r="C24" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D24" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="7"/>
+      <c r="C25" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="206" t="s">
+        <v>70</v>
+      </c>
+      <c r="C26" s="201"/>
+      <c r="D26" s="201"/>
+      <c r="E26" s="201"/>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="205" t="s">
+        <v>71</v>
+      </c>
+      <c r="C28" s="201"/>
+      <c r="D28" s="201"/>
+      <c r="E28" s="201"/>
+    </row>
+    <row r="29" spans="2:5" ht="36" x14ac:dyDescent="0.25">
+      <c r="B29" s="30"/>
+      <c r="C29" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D29" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" ht="36" x14ac:dyDescent="0.25">
+      <c r="C30" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D30" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="203" t="s">
+        <v>78</v>
+      </c>
+      <c r="C31" s="201"/>
+      <c r="D31" s="201"/>
+      <c r="E31" s="201"/>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B32" s="201"/>
+      <c r="C32" s="201"/>
+      <c r="D32" s="201"/>
+      <c r="E32" s="201"/>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B34" s="205" t="s">
+        <v>79</v>
+      </c>
+      <c r="C34" s="201"/>
+      <c r="D34" s="201"/>
+      <c r="E34" s="201"/>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B35" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" ht="39" x14ac:dyDescent="0.25">
+      <c r="B36" s="210" t="s">
+        <v>198</v>
+      </c>
+      <c r="C36" s="31" t="s">
+        <v>197</v>
+      </c>
+      <c r="D36" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="36" x14ac:dyDescent="0.25">
-      <c r="A17" s="174"/>
-      <c r="B17" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C17" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="A18" s="175"/>
-      <c r="B18" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="C18" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="A19" s="176"/>
-      <c r="B19" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="A20" s="26"/>
-      <c r="B20" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C20" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="A21" s="27"/>
-      <c r="B21" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C21" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="36" x14ac:dyDescent="0.25">
-      <c r="A22" s="162"/>
-      <c r="B22" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C22" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="36" x14ac:dyDescent="0.25">
-      <c r="A23" s="28"/>
-      <c r="B23" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="A24" s="29"/>
-      <c r="B24" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C24" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="7"/>
-      <c r="B25" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C25" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="203" t="s">
-        <v>70</v>
-      </c>
-      <c r="B26" s="196"/>
-      <c r="C26" s="196"/>
-      <c r="D26" s="196"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="202" t="s">
-        <v>71</v>
-      </c>
-      <c r="B28" s="196"/>
-      <c r="C28" s="196"/>
-      <c r="D28" s="196"/>
-    </row>
-    <row r="29" spans="1:4" ht="36" x14ac:dyDescent="0.25">
-      <c r="A29" s="30"/>
-      <c r="B29" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C29" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="36" x14ac:dyDescent="0.25">
-      <c r="B30" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C30" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="200" t="s">
-        <v>78</v>
-      </c>
-      <c r="B31" s="196"/>
-      <c r="C31" s="196"/>
-      <c r="D31" s="196"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="196"/>
-      <c r="B32" s="196"/>
-      <c r="C32" s="196"/>
-      <c r="D32" s="196"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="202" t="s">
-        <v>79</v>
-      </c>
-      <c r="B34" s="196"/>
-      <c r="C34" s="196"/>
-      <c r="D34" s="196"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="31" t="s">
+    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B37" s="211"/>
+      <c r="C37" s="32"/>
+      <c r="D37" s="32"/>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B38" s="211"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B39" s="211"/>
+      <c r="C39" s="32"/>
+      <c r="D39" s="32"/>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B40" s="211"/>
+      <c r="C40" s="32"/>
+      <c r="D40" s="32"/>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B41" s="211"/>
+      <c r="C41" s="32"/>
+      <c r="D41" s="32"/>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B42" s="211"/>
+      <c r="C42" s="32"/>
+      <c r="D42" s="32"/>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B43" s="211"/>
+      <c r="C43" s="32"/>
+      <c r="D43" s="32"/>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B44" s="211"/>
+      <c r="C44" s="32"/>
+      <c r="D44" s="32"/>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B45" s="211"/>
+      <c r="C45" s="32"/>
+      <c r="D45" s="32"/>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B46" s="211"/>
+      <c r="C46" s="32"/>
+      <c r="D46" s="32"/>
+    </row>
+    <row r="47" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B47" s="211"/>
+      <c r="C47" s="32"/>
+      <c r="D47" s="32"/>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B48" s="211"/>
+      <c r="C48" s="32"/>
+      <c r="D48" s="32"/>
+    </row>
+    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B49" s="211"/>
+      <c r="C49" s="32"/>
+      <c r="D49" s="32"/>
+    </row>
+    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B50" s="211"/>
+      <c r="C50" s="32"/>
+      <c r="D50" s="32"/>
+    </row>
+    <row r="51" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B51" s="203" t="s">
         <v>83</v>
       </c>
-      <c r="B36" s="31" t="s">
+      <c r="C51" s="201"/>
+      <c r="D51" s="201"/>
+      <c r="E51" s="201"/>
+    </row>
+    <row r="52" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B52" s="201"/>
+      <c r="C52" s="201"/>
+      <c r="D52" s="201"/>
+      <c r="E52" s="201"/>
+    </row>
+    <row r="56" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B56" s="207" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="32"/>
-      <c r="B37" s="32"/>
-      <c r="C37" s="32"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="32"/>
-      <c r="B38" s="32"/>
-      <c r="C38" s="32"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="32"/>
-      <c r="B39" s="32"/>
-      <c r="C39" s="32"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="32"/>
-      <c r="B40" s="32"/>
-      <c r="C40" s="32"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="32"/>
-      <c r="B41" s="32"/>
-      <c r="C41" s="32"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="32"/>
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="32"/>
-      <c r="B43" s="32"/>
-      <c r="C43" s="32"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="32"/>
-      <c r="B44" s="32"/>
-      <c r="C44" s="32"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="32"/>
-      <c r="B45" s="32"/>
-      <c r="C45" s="32"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="32"/>
-      <c r="B46" s="32"/>
-      <c r="C46" s="32"/>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="32"/>
-      <c r="B47" s="32"/>
-      <c r="C47" s="32"/>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="32"/>
-      <c r="B48" s="32"/>
-      <c r="C48" s="32"/>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="32"/>
-      <c r="B49" s="32"/>
-      <c r="C49" s="32"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="32"/>
-      <c r="B50" s="32"/>
-      <c r="C50" s="32"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="200" t="s">
+      <c r="C56" s="201"/>
+      <c r="D56" s="201"/>
+      <c r="E56" s="201"/>
+    </row>
+    <row r="57" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B57" s="200" t="s">
         <v>85</v>
       </c>
-      <c r="B51" s="196"/>
-      <c r="C51" s="196"/>
-      <c r="D51" s="196"/>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="196"/>
-      <c r="B52" s="196"/>
-      <c r="C52" s="196"/>
-      <c r="D52" s="196"/>
-    </row>
-    <row r="56" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="199" t="s">
+      <c r="C57" s="201"/>
+      <c r="D57" s="201"/>
+      <c r="E57" s="201"/>
+    </row>
+    <row r="58" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B58" s="200" t="s">
         <v>86</v>
       </c>
-      <c r="B56" s="196"/>
-      <c r="C56" s="196"/>
-      <c r="D56" s="196"/>
-    </row>
-    <row r="57" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="198" t="s">
+      <c r="C58" s="201"/>
+      <c r="D58" s="201"/>
+      <c r="E58" s="201"/>
+    </row>
+    <row r="59" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B59" s="200" t="s">
         <v>87</v>
       </c>
-      <c r="B57" s="196"/>
-      <c r="C57" s="196"/>
-      <c r="D57" s="196"/>
-    </row>
-    <row r="58" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="198" t="s">
+      <c r="C59" s="201"/>
+      <c r="D59" s="201"/>
+      <c r="E59" s="201"/>
+    </row>
+    <row r="60" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B60" s="200" t="s">
         <v>88</v>
       </c>
-      <c r="B58" s="196"/>
-      <c r="C58" s="196"/>
-      <c r="D58" s="196"/>
-    </row>
-    <row r="59" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="198" t="s">
+      <c r="C60" s="201"/>
+      <c r="D60" s="201"/>
+      <c r="E60" s="201"/>
+    </row>
+    <row r="61" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B61" s="200" t="s">
         <v>89</v>
       </c>
-      <c r="B59" s="196"/>
-      <c r="C59" s="196"/>
-      <c r="D59" s="196"/>
-    </row>
-    <row r="60" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="198" t="s">
+      <c r="C61" s="201"/>
+      <c r="D61" s="201"/>
+      <c r="E61" s="201"/>
+    </row>
+    <row r="62" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B62" s="200" t="s">
         <v>90</v>
       </c>
-      <c r="B60" s="196"/>
-      <c r="C60" s="196"/>
-      <c r="D60" s="196"/>
-    </row>
-    <row r="61" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="198" t="s">
+      <c r="C62" s="201"/>
+      <c r="D62" s="201"/>
+      <c r="E62" s="201"/>
+    </row>
+    <row r="63" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B63" s="200" t="s">
         <v>91</v>
       </c>
-      <c r="B61" s="196"/>
-      <c r="C61" s="196"/>
-      <c r="D61" s="196"/>
-    </row>
-    <row r="62" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="198" t="s">
+      <c r="C63" s="201"/>
+      <c r="D63" s="201"/>
+      <c r="E63" s="201"/>
+    </row>
+    <row r="64" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B64" s="200" t="s">
         <v>92</v>
       </c>
-      <c r="B62" s="196"/>
-      <c r="C62" s="196"/>
-      <c r="D62" s="196"/>
-    </row>
-    <row r="63" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="198" t="s">
+      <c r="C64" s="201"/>
+      <c r="D64" s="201"/>
+      <c r="E64" s="201"/>
+    </row>
+    <row r="65" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B65" s="200" t="s">
         <v>93</v>
       </c>
-      <c r="B63" s="196"/>
-      <c r="C63" s="196"/>
-      <c r="D63" s="196"/>
-    </row>
-    <row r="64" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="198" t="s">
+      <c r="C65" s="201"/>
+      <c r="D65" s="201"/>
+      <c r="E65" s="201"/>
+    </row>
+    <row r="66" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B66" s="200" t="s">
         <v>94</v>
       </c>
-      <c r="B64" s="196"/>
-      <c r="C64" s="196"/>
-      <c r="D64" s="196"/>
-    </row>
-    <row r="65" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="198" t="s">
+      <c r="C66" s="201"/>
+      <c r="D66" s="201"/>
+      <c r="E66" s="201"/>
+    </row>
+    <row r="67" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B67" s="200" t="s">
         <v>95</v>
       </c>
-      <c r="B65" s="196"/>
-      <c r="C65" s="196"/>
-      <c r="D65" s="196"/>
-    </row>
-    <row r="66" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="198" t="s">
+      <c r="C67" s="201"/>
+      <c r="D67" s="201"/>
+      <c r="E67" s="201"/>
+    </row>
+    <row r="68" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B68" s="200"/>
+      <c r="C68" s="201"/>
+      <c r="D68" s="201"/>
+      <c r="E68" s="201"/>
+    </row>
+    <row r="69" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B69" s="207" t="s">
         <v>96</v>
       </c>
-      <c r="B66" s="196"/>
-      <c r="C66" s="196"/>
-      <c r="D66" s="196"/>
-    </row>
-    <row r="67" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="198" t="s">
+      <c r="C69" s="201"/>
+      <c r="D69" s="201"/>
+      <c r="E69" s="201"/>
+    </row>
+    <row r="70" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B70" s="200" t="s">
         <v>97</v>
       </c>
-      <c r="B67" s="196"/>
-      <c r="C67" s="196"/>
-      <c r="D67" s="196"/>
-    </row>
-    <row r="68" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="198"/>
-      <c r="B68" s="196"/>
-      <c r="C68" s="196"/>
-      <c r="D68" s="196"/>
-    </row>
-    <row r="69" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="199" t="s">
+      <c r="C70" s="201"/>
+      <c r="D70" s="201"/>
+      <c r="E70" s="201"/>
+    </row>
+    <row r="71" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B71" s="200" t="s">
         <v>98</v>
       </c>
-      <c r="B69" s="196"/>
-      <c r="C69" s="196"/>
-      <c r="D69" s="196"/>
-    </row>
-    <row r="70" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="198" t="s">
+      <c r="C71" s="201"/>
+      <c r="D71" s="201"/>
+      <c r="E71" s="201"/>
+    </row>
+    <row r="72" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B72" s="200" t="s">
         <v>99</v>
       </c>
-      <c r="B70" s="196"/>
-      <c r="C70" s="196"/>
-      <c r="D70" s="196"/>
-    </row>
-    <row r="71" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="198" t="s">
+      <c r="C72" s="201"/>
+      <c r="D72" s="201"/>
+      <c r="E72" s="201"/>
+    </row>
+    <row r="73" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B73" s="200" t="s">
         <v>100</v>
       </c>
-      <c r="B71" s="196"/>
-      <c r="C71" s="196"/>
-      <c r="D71" s="196"/>
-    </row>
-    <row r="72" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="198" t="s">
+      <c r="C73" s="201"/>
+      <c r="D73" s="201"/>
+      <c r="E73" s="201"/>
+    </row>
+    <row r="74" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B74" s="200" t="s">
         <v>101</v>
       </c>
-      <c r="B72" s="196"/>
-      <c r="C72" s="196"/>
-      <c r="D72" s="196"/>
-    </row>
-    <row r="73" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="198" t="s">
+      <c r="C74" s="201"/>
+      <c r="D74" s="201"/>
+      <c r="E74" s="201"/>
+    </row>
+    <row r="75" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B75" s="200" t="s">
         <v>102</v>
       </c>
-      <c r="B73" s="196"/>
-      <c r="C73" s="196"/>
-      <c r="D73" s="196"/>
-    </row>
-    <row r="74" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="198" t="s">
+      <c r="C75" s="201"/>
+      <c r="D75" s="201"/>
+      <c r="E75" s="201"/>
+    </row>
+    <row r="76" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B76" s="200"/>
+      <c r="C76" s="201"/>
+      <c r="D76" s="201"/>
+      <c r="E76" s="201"/>
+    </row>
+    <row r="77" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B77" s="207" t="s">
         <v>103</v>
       </c>
-      <c r="B74" s="196"/>
-      <c r="C74" s="196"/>
-      <c r="D74" s="196"/>
-    </row>
-    <row r="75" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="198" t="s">
+      <c r="C77" s="201"/>
+      <c r="D77" s="201"/>
+      <c r="E77" s="201"/>
+    </row>
+    <row r="78" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B78" s="200" t="s">
         <v>104</v>
       </c>
-      <c r="B75" s="196"/>
-      <c r="C75" s="196"/>
-      <c r="D75" s="196"/>
-    </row>
-    <row r="76" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="198"/>
-      <c r="B76" s="196"/>
-      <c r="C76" s="196"/>
-      <c r="D76" s="196"/>
-    </row>
-    <row r="77" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="199" t="s">
+      <c r="C78" s="201"/>
+      <c r="D78" s="201"/>
+      <c r="E78" s="201"/>
+    </row>
+    <row r="79" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B79" s="200" t="s">
         <v>105</v>
       </c>
-      <c r="B77" s="196"/>
-      <c r="C77" s="196"/>
-      <c r="D77" s="196"/>
-    </row>
-    <row r="78" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="198" t="s">
+      <c r="C79" s="201"/>
+      <c r="D79" s="201"/>
+      <c r="E79" s="201"/>
+    </row>
+    <row r="80" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B80" s="200" t="s">
         <v>106</v>
       </c>
-      <c r="B78" s="196"/>
-      <c r="C78" s="196"/>
-      <c r="D78" s="196"/>
-    </row>
-    <row r="79" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="198" t="s">
+      <c r="C80" s="201"/>
+      <c r="D80" s="201"/>
+      <c r="E80" s="201"/>
+    </row>
+    <row r="81" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B81" s="200" t="s">
         <v>107</v>
       </c>
-      <c r="B79" s="196"/>
-      <c r="C79" s="196"/>
-      <c r="D79" s="196"/>
-    </row>
-    <row r="80" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="198" t="s">
+      <c r="C81" s="201"/>
+      <c r="D81" s="201"/>
+      <c r="E81" s="201"/>
+    </row>
+    <row r="82" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B82" s="200" t="s">
         <v>108</v>
       </c>
-      <c r="B80" s="196"/>
-      <c r="C80" s="196"/>
-      <c r="D80" s="196"/>
-    </row>
-    <row r="81" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="198" t="s">
+      <c r="C82" s="201"/>
+      <c r="D82" s="201"/>
+      <c r="E82" s="201"/>
+    </row>
+    <row r="83" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B83" s="200"/>
+      <c r="C83" s="201"/>
+      <c r="D83" s="201"/>
+      <c r="E83" s="201"/>
+    </row>
+    <row r="84" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B84" s="207" t="s">
         <v>109</v>
       </c>
-      <c r="B81" s="196"/>
-      <c r="C81" s="196"/>
-      <c r="D81" s="196"/>
-    </row>
-    <row r="82" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="198" t="s">
+      <c r="C84" s="201"/>
+      <c r="D84" s="201"/>
+      <c r="E84" s="201"/>
+    </row>
+    <row r="85" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B85" s="200" t="s">
         <v>110</v>
       </c>
-      <c r="B82" s="196"/>
-      <c r="C82" s="196"/>
-      <c r="D82" s="196"/>
-    </row>
-    <row r="83" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="198"/>
-      <c r="B83" s="196"/>
-      <c r="C83" s="196"/>
-      <c r="D83" s="196"/>
-    </row>
-    <row r="84" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="199" t="s">
+      <c r="C85" s="201"/>
+      <c r="D85" s="201"/>
+      <c r="E85" s="201"/>
+    </row>
+    <row r="86" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B86" s="200" t="s">
         <v>111</v>
       </c>
-      <c r="B84" s="196"/>
-      <c r="C84" s="196"/>
-      <c r="D84" s="196"/>
-    </row>
-    <row r="85" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="198" t="s">
+      <c r="C86" s="201"/>
+      <c r="D86" s="201"/>
+      <c r="E86" s="201"/>
+    </row>
+    <row r="87" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B87" s="200" t="s">
         <v>112</v>
       </c>
-      <c r="B85" s="196"/>
-      <c r="C85" s="196"/>
-      <c r="D85" s="196"/>
-    </row>
-    <row r="86" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="198" t="s">
+      <c r="C87" s="201"/>
+      <c r="D87" s="201"/>
+      <c r="E87" s="201"/>
+    </row>
+    <row r="88" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B88" s="200" t="s">
         <v>113</v>
       </c>
-      <c r="B86" s="196"/>
-      <c r="C86" s="196"/>
-      <c r="D86" s="196"/>
-    </row>
-    <row r="87" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="198" t="s">
+      <c r="C88" s="201"/>
+      <c r="D88" s="201"/>
+      <c r="E88" s="201"/>
+    </row>
+    <row r="89" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B89" s="200" t="s">
         <v>114</v>
       </c>
-      <c r="B87" s="196"/>
-      <c r="C87" s="196"/>
-      <c r="D87" s="196"/>
-    </row>
-    <row r="88" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="198" t="s">
+      <c r="C89" s="201"/>
+      <c r="D89" s="201"/>
+      <c r="E89" s="201"/>
+    </row>
+    <row r="90" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B90" s="200" t="s">
         <v>115</v>
       </c>
-      <c r="B88" s="196"/>
-      <c r="C88" s="196"/>
-      <c r="D88" s="196"/>
-    </row>
-    <row r="89" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="198" t="s">
+      <c r="C90" s="201"/>
+      <c r="D90" s="201"/>
+      <c r="E90" s="201"/>
+    </row>
+    <row r="91" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B91" s="200" t="s">
         <v>116</v>
       </c>
-      <c r="B89" s="196"/>
-      <c r="C89" s="196"/>
-      <c r="D89" s="196"/>
-    </row>
-    <row r="90" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="198" t="s">
+      <c r="C91" s="201"/>
+      <c r="D91" s="201"/>
+      <c r="E91" s="201"/>
+    </row>
+    <row r="92" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B92" s="200"/>
+      <c r="C92" s="201"/>
+      <c r="D92" s="201"/>
+      <c r="E92" s="201"/>
+    </row>
+    <row r="93" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B93" s="207" t="s">
         <v>117</v>
       </c>
-      <c r="B90" s="196"/>
-      <c r="C90" s="196"/>
-      <c r="D90" s="196"/>
-    </row>
-    <row r="91" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="198" t="s">
+      <c r="C93" s="201"/>
+      <c r="D93" s="201"/>
+      <c r="E93" s="201"/>
+    </row>
+    <row r="94" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B94" s="200" t="s">
         <v>118</v>
       </c>
-      <c r="B91" s="196"/>
-      <c r="C91" s="196"/>
-      <c r="D91" s="196"/>
-    </row>
-    <row r="92" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="198"/>
-      <c r="B92" s="196"/>
-      <c r="C92" s="196"/>
-      <c r="D92" s="196"/>
-    </row>
-    <row r="93" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="199" t="s">
+      <c r="C94" s="201"/>
+      <c r="D94" s="201"/>
+      <c r="E94" s="201"/>
+    </row>
+    <row r="95" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B95" s="200" t="s">
         <v>119</v>
       </c>
-      <c r="B93" s="196"/>
-      <c r="C93" s="196"/>
-      <c r="D93" s="196"/>
-    </row>
-    <row r="94" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="198" t="s">
+      <c r="C95" s="201"/>
+      <c r="D95" s="201"/>
+      <c r="E95" s="201"/>
+    </row>
+    <row r="96" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B96" s="200" t="s">
         <v>120</v>
       </c>
-      <c r="B94" s="196"/>
-      <c r="C94" s="196"/>
-      <c r="D94" s="196"/>
-    </row>
-    <row r="95" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="198" t="s">
+      <c r="C96" s="201"/>
+      <c r="D96" s="201"/>
+      <c r="E96" s="201"/>
+    </row>
+    <row r="97" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B97" s="200" t="s">
         <v>121</v>
       </c>
-      <c r="B95" s="196"/>
-      <c r="C95" s="196"/>
-      <c r="D95" s="196"/>
-    </row>
-    <row r="96" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="198" t="s">
+      <c r="C97" s="201"/>
+      <c r="D97" s="201"/>
+      <c r="E97" s="201"/>
+    </row>
+    <row r="98" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B98" s="200" t="s">
         <v>122</v>
       </c>
-      <c r="B96" s="196"/>
-      <c r="C96" s="196"/>
-      <c r="D96" s="196"/>
-    </row>
-    <row r="97" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="198" t="s">
+      <c r="C98" s="201"/>
+      <c r="D98" s="201"/>
+      <c r="E98" s="201"/>
+    </row>
+    <row r="99" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B99" s="200" t="s">
         <v>123</v>
       </c>
-      <c r="B97" s="196"/>
-      <c r="C97" s="196"/>
-      <c r="D97" s="196"/>
-    </row>
-    <row r="98" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="198" t="s">
-        <v>124</v>
-      </c>
-      <c r="B98" s="196"/>
-      <c r="C98" s="196"/>
-      <c r="D98" s="196"/>
-    </row>
-    <row r="99" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="198" t="s">
-        <v>125</v>
-      </c>
-      <c r="B99" s="196"/>
-      <c r="C99" s="196"/>
-      <c r="D99" s="196"/>
+      <c r="C99" s="201"/>
+      <c r="D99" s="201"/>
+      <c r="E99" s="201"/>
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="A60:D60"/>
-    <mergeCell ref="A61:D61"/>
-    <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A66:D66"/>
-    <mergeCell ref="A74:D74"/>
-    <mergeCell ref="A68:D68"/>
-    <mergeCell ref="A63:D63"/>
-    <mergeCell ref="A86:D86"/>
-    <mergeCell ref="A64:D64"/>
-    <mergeCell ref="A79:D79"/>
-    <mergeCell ref="A83:D83"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A51:D52"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A3:D5"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="A31:D32"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A65:D65"/>
-    <mergeCell ref="A92:D92"/>
-    <mergeCell ref="A73:D73"/>
-    <mergeCell ref="A82:D82"/>
-    <mergeCell ref="A91:D91"/>
-    <mergeCell ref="A69:D69"/>
-    <mergeCell ref="A88:D88"/>
-    <mergeCell ref="A70:D70"/>
-    <mergeCell ref="A84:D84"/>
-    <mergeCell ref="A90:D90"/>
-    <mergeCell ref="A72:D72"/>
-    <mergeCell ref="A71:D71"/>
-    <mergeCell ref="A77:D77"/>
-    <mergeCell ref="A85:D85"/>
-    <mergeCell ref="A67:D67"/>
-    <mergeCell ref="A78:D78"/>
-    <mergeCell ref="A99:D99"/>
-    <mergeCell ref="A75:D75"/>
-    <mergeCell ref="A89:D89"/>
-    <mergeCell ref="A80:D80"/>
-    <mergeCell ref="A97:D97"/>
-    <mergeCell ref="A81:D81"/>
-    <mergeCell ref="A87:D87"/>
-    <mergeCell ref="A96:D96"/>
-    <mergeCell ref="A98:D98"/>
-    <mergeCell ref="A94:D94"/>
-    <mergeCell ref="A95:D95"/>
-    <mergeCell ref="A76:D76"/>
-    <mergeCell ref="A93:D93"/>
+    <mergeCell ref="B99:E99"/>
+    <mergeCell ref="B75:E75"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="B80:E80"/>
+    <mergeCell ref="B97:E97"/>
+    <mergeCell ref="B81:E81"/>
+    <mergeCell ref="B87:E87"/>
+    <mergeCell ref="B96:E96"/>
+    <mergeCell ref="B98:E98"/>
+    <mergeCell ref="B94:E94"/>
+    <mergeCell ref="B95:E95"/>
+    <mergeCell ref="B76:E76"/>
+    <mergeCell ref="B93:E93"/>
+    <mergeCell ref="B92:E92"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="B82:E82"/>
+    <mergeCell ref="B91:E91"/>
+    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="B88:E88"/>
+    <mergeCell ref="B70:E70"/>
+    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="B90:E90"/>
+    <mergeCell ref="B72:E72"/>
+    <mergeCell ref="B71:E71"/>
+    <mergeCell ref="B77:E77"/>
+    <mergeCell ref="B85:E85"/>
+    <mergeCell ref="B78:E78"/>
+    <mergeCell ref="B86:E86"/>
+    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="B79:E79"/>
+    <mergeCell ref="B83:E83"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B51:E52"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="B3:E5"/>
+    <mergeCell ref="B59:E59"/>
+    <mergeCell ref="B31:E32"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B57:E57"/>
+    <mergeCell ref="B56:E56"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="B62:E62"/>
+    <mergeCell ref="B66:E66"/>
+    <mergeCell ref="B74:E74"/>
+    <mergeCell ref="B68:E68"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="B65:E65"/>
+    <mergeCell ref="B67:E67"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11663,84 +11651,84 @@
       <c r="BI61" s="8"/>
     </row>
     <row r="63" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A63" s="204" t="s">
+      <c r="A63" s="209" t="s">
         <v>15</v>
       </c>
-      <c r="B63" s="196"/>
-      <c r="C63" s="196"/>
-      <c r="D63" s="196"/>
-      <c r="E63" s="196"/>
-      <c r="F63" s="196"/>
-      <c r="G63" s="196"/>
-      <c r="H63" s="196"/>
-      <c r="I63" s="196"/>
-      <c r="J63" s="196"/>
-      <c r="K63" s="196"/>
-      <c r="L63" s="196"/>
-      <c r="M63" s="196"/>
-      <c r="N63" s="196"/>
-      <c r="O63" s="196"/>
-      <c r="P63" s="196"/>
-      <c r="Q63" s="196"/>
-      <c r="R63" s="196"/>
-      <c r="S63" s="196"/>
-      <c r="T63" s="196"/>
-      <c r="U63" s="196"/>
-      <c r="V63" s="196"/>
-      <c r="W63" s="196"/>
-      <c r="X63" s="196"/>
+      <c r="B63" s="201"/>
+      <c r="C63" s="201"/>
+      <c r="D63" s="201"/>
+      <c r="E63" s="201"/>
+      <c r="F63" s="201"/>
+      <c r="G63" s="201"/>
+      <c r="H63" s="201"/>
+      <c r="I63" s="201"/>
+      <c r="J63" s="201"/>
+      <c r="K63" s="201"/>
+      <c r="L63" s="201"/>
+      <c r="M63" s="201"/>
+      <c r="N63" s="201"/>
+      <c r="O63" s="201"/>
+      <c r="P63" s="201"/>
+      <c r="Q63" s="201"/>
+      <c r="R63" s="201"/>
+      <c r="S63" s="201"/>
+      <c r="T63" s="201"/>
+      <c r="U63" s="201"/>
+      <c r="V63" s="201"/>
+      <c r="W63" s="201"/>
+      <c r="X63" s="201"/>
     </row>
     <row r="64" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A64" s="196"/>
-      <c r="B64" s="196"/>
-      <c r="C64" s="196"/>
-      <c r="D64" s="196"/>
-      <c r="E64" s="196"/>
-      <c r="F64" s="196"/>
-      <c r="G64" s="196"/>
-      <c r="H64" s="196"/>
-      <c r="I64" s="196"/>
-      <c r="J64" s="196"/>
-      <c r="K64" s="196"/>
-      <c r="L64" s="196"/>
-      <c r="M64" s="196"/>
-      <c r="N64" s="196"/>
-      <c r="O64" s="196"/>
-      <c r="P64" s="196"/>
-      <c r="Q64" s="196"/>
-      <c r="R64" s="196"/>
-      <c r="S64" s="196"/>
-      <c r="T64" s="196"/>
-      <c r="U64" s="196"/>
-      <c r="V64" s="196"/>
-      <c r="W64" s="196"/>
-      <c r="X64" s="196"/>
+      <c r="A64" s="201"/>
+      <c r="B64" s="201"/>
+      <c r="C64" s="201"/>
+      <c r="D64" s="201"/>
+      <c r="E64" s="201"/>
+      <c r="F64" s="201"/>
+      <c r="G64" s="201"/>
+      <c r="H64" s="201"/>
+      <c r="I64" s="201"/>
+      <c r="J64" s="201"/>
+      <c r="K64" s="201"/>
+      <c r="L64" s="201"/>
+      <c r="M64" s="201"/>
+      <c r="N64" s="201"/>
+      <c r="O64" s="201"/>
+      <c r="P64" s="201"/>
+      <c r="Q64" s="201"/>
+      <c r="R64" s="201"/>
+      <c r="S64" s="201"/>
+      <c r="T64" s="201"/>
+      <c r="U64" s="201"/>
+      <c r="V64" s="201"/>
+      <c r="W64" s="201"/>
+      <c r="X64" s="201"/>
     </row>
     <row r="65" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A65" s="196"/>
-      <c r="B65" s="196"/>
-      <c r="C65" s="196"/>
-      <c r="D65" s="196"/>
-      <c r="E65" s="196"/>
-      <c r="F65" s="196"/>
-      <c r="G65" s="196"/>
-      <c r="H65" s="196"/>
-      <c r="I65" s="196"/>
-      <c r="J65" s="196"/>
-      <c r="K65" s="196"/>
-      <c r="L65" s="196"/>
-      <c r="M65" s="196"/>
-      <c r="N65" s="196"/>
-      <c r="O65" s="196"/>
-      <c r="P65" s="196"/>
-      <c r="Q65" s="196"/>
-      <c r="R65" s="196"/>
-      <c r="S65" s="196"/>
-      <c r="T65" s="196"/>
-      <c r="U65" s="196"/>
-      <c r="V65" s="196"/>
-      <c r="W65" s="196"/>
-      <c r="X65" s="196"/>
+      <c r="A65" s="201"/>
+      <c r="B65" s="201"/>
+      <c r="C65" s="201"/>
+      <c r="D65" s="201"/>
+      <c r="E65" s="201"/>
+      <c r="F65" s="201"/>
+      <c r="G65" s="201"/>
+      <c r="H65" s="201"/>
+      <c r="I65" s="201"/>
+      <c r="J65" s="201"/>
+      <c r="K65" s="201"/>
+      <c r="L65" s="201"/>
+      <c r="M65" s="201"/>
+      <c r="N65" s="201"/>
+      <c r="O65" s="201"/>
+      <c r="P65" s="201"/>
+      <c r="Q65" s="201"/>
+      <c r="R65" s="201"/>
+      <c r="S65" s="201"/>
+      <c r="T65" s="201"/>
+      <c r="U65" s="201"/>
+      <c r="V65" s="201"/>
+      <c r="W65" s="201"/>
+      <c r="X65" s="201"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11762,12 +11750,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="195" t="s">
+      <c r="A1" s="202" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="196"/>
-      <c r="C1" s="196"/>
-      <c r="D1" s="196"/>
+      <c r="B1" s="201"/>
+      <c r="C1" s="201"/>
+      <c r="D1" s="201"/>
     </row>
     <row r="3" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
@@ -11825,7 +11813,7 @@
         <v>28</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>29</v>
@@ -11837,7 +11825,7 @@
         <v>30</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>31</v>
@@ -11861,7 +11849,7 @@
         <v>34</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>35</v>
@@ -11892,18 +11880,18 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="204" t="s">
+      <c r="A14" s="209" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="196"/>
-      <c r="C14" s="196"/>
-      <c r="D14" s="196"/>
+      <c r="B14" s="201"/>
+      <c r="C14" s="201"/>
+      <c r="D14" s="201"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="196"/>
-      <c r="B15" s="196"/>
-      <c r="C15" s="196"/>
-      <c r="D15" s="196"/>
+      <c r="A15" s="201"/>
+      <c r="B15" s="201"/>
+      <c r="C15" s="201"/>
+      <c r="D15" s="201"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="161"/>
@@ -11929,187 +11917,187 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="195" t="s">
-        <v>198</v>
-      </c>
-      <c r="B1" s="196"/>
-      <c r="C1" s="196"/>
-      <c r="D1" s="196"/>
+      <c r="A1" s="202" t="s">
+        <v>193</v>
+      </c>
+      <c r="B1" s="201"/>
+      <c r="C1" s="201"/>
+      <c r="D1" s="201"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="197" t="s">
-        <v>197</v>
-      </c>
-      <c r="B2" s="196"/>
-      <c r="C2" s="196"/>
-      <c r="D2" s="196"/>
+      <c r="A2" s="208" t="s">
+        <v>192</v>
+      </c>
+      <c r="B2" s="201"/>
+      <c r="C2" s="201"/>
+      <c r="D2" s="201"/>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="207" t="s">
-        <v>192</v>
-      </c>
-      <c r="B5" s="206" t="s">
-        <v>191</v>
-      </c>
-      <c r="C5" s="205" t="s">
-        <v>190</v>
-      </c>
-      <c r="D5" s="205" t="s">
-        <v>189</v>
+      <c r="A5" s="197" t="s">
+        <v>187</v>
+      </c>
+      <c r="B5" s="196" t="s">
+        <v>186</v>
+      </c>
+      <c r="C5" s="195" t="s">
+        <v>185</v>
+      </c>
+      <c r="D5" s="195" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="207" t="s">
-        <v>188</v>
-      </c>
-      <c r="B6" s="206" t="s">
-        <v>187</v>
-      </c>
-      <c r="C6" s="205" t="s">
-        <v>186</v>
-      </c>
-      <c r="D6" s="205" t="s">
-        <v>185</v>
+      <c r="A6" s="197" t="s">
+        <v>183</v>
+      </c>
+      <c r="B6" s="196" t="s">
+        <v>182</v>
+      </c>
+      <c r="C6" s="195" t="s">
+        <v>181</v>
+      </c>
+      <c r="D6" s="195" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="207" t="s">
+      <c r="A7" s="197" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="206" t="s">
+      <c r="B7" s="196" t="s">
+        <v>168</v>
+      </c>
+      <c r="C7" s="195" t="s">
+        <v>179</v>
+      </c>
+      <c r="D7" s="195" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="197" t="s">
+        <v>177</v>
+      </c>
+      <c r="B8" s="196" t="s">
+        <v>158</v>
+      </c>
+      <c r="C8" s="195" t="s">
+        <v>176</v>
+      </c>
+      <c r="D8" s="195" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="197" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="196" t="s">
+        <v>168</v>
+      </c>
+      <c r="C9" s="195" t="s">
+        <v>174</v>
+      </c>
+      <c r="D9" s="195" t="s">
         <v>173</v>
       </c>
-      <c r="C7" s="205" t="s">
-        <v>184</v>
-      </c>
-      <c r="D7" s="205" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="207" t="s">
-        <v>182</v>
-      </c>
-      <c r="B8" s="206" t="s">
+    </row>
+    <row r="10" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="197" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="196" t="s">
+        <v>172</v>
+      </c>
+      <c r="C10" s="195" t="s">
+        <v>171</v>
+      </c>
+      <c r="D10" s="195" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="197" t="s">
+        <v>169</v>
+      </c>
+      <c r="B11" s="196" t="s">
+        <v>168</v>
+      </c>
+      <c r="C11" s="195" t="s">
+        <v>167</v>
+      </c>
+      <c r="D11" s="195" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="197" t="s">
+        <v>150</v>
+      </c>
+      <c r="B12" s="196" t="s">
+        <v>158</v>
+      </c>
+      <c r="C12" s="195" t="s">
+        <v>165</v>
+      </c>
+      <c r="D12" s="195" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="197" t="s">
+        <v>152</v>
+      </c>
+      <c r="B13" s="196" t="s">
+        <v>158</v>
+      </c>
+      <c r="C13" s="195" t="s">
         <v>163</v>
       </c>
-      <c r="C8" s="205" t="s">
-        <v>181</v>
-      </c>
-      <c r="D8" s="205" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="207" t="s">
-        <v>58</v>
-      </c>
-      <c r="B9" s="206" t="s">
-        <v>173</v>
-      </c>
-      <c r="C9" s="205" t="s">
-        <v>179</v>
-      </c>
-      <c r="D9" s="205" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="207" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" s="206" t="s">
-        <v>177</v>
-      </c>
-      <c r="C10" s="205" t="s">
-        <v>176</v>
-      </c>
-      <c r="D10" s="205" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="207" t="s">
-        <v>174</v>
-      </c>
-      <c r="B11" s="206" t="s">
-        <v>173</v>
-      </c>
-      <c r="C11" s="205" t="s">
-        <v>172</v>
-      </c>
-      <c r="D11" s="205" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="207" t="s">
-        <v>155</v>
-      </c>
-      <c r="B12" s="206" t="s">
-        <v>163</v>
-      </c>
-      <c r="C12" s="205" t="s">
-        <v>170</v>
-      </c>
-      <c r="D12" s="205" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="207" t="s">
+      <c r="D13" s="195" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="197" t="s">
+        <v>154</v>
+      </c>
+      <c r="B14" s="196" t="s">
+        <v>158</v>
+      </c>
+      <c r="C14" s="195" t="s">
+        <v>161</v>
+      </c>
+      <c r="D14" s="195" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="197" t="s">
+        <v>159</v>
+      </c>
+      <c r="B15" s="196" t="s">
+        <v>158</v>
+      </c>
+      <c r="C15" s="195" t="s">
         <v>157</v>
       </c>
-      <c r="B13" s="206" t="s">
-        <v>163</v>
-      </c>
-      <c r="C13" s="205" t="s">
-        <v>168</v>
-      </c>
-      <c r="D13" s="205" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="207" t="s">
-        <v>159</v>
-      </c>
-      <c r="B14" s="206" t="s">
-        <v>163</v>
-      </c>
-      <c r="C14" s="205" t="s">
-        <v>166</v>
-      </c>
-      <c r="D14" s="205" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="207" t="s">
-        <v>164</v>
-      </c>
-      <c r="B15" s="206" t="s">
-        <v>163</v>
-      </c>
-      <c r="C15" s="205" t="s">
-        <v>162</v>
-      </c>
-      <c r="D15" s="205" t="s">
-        <v>161</v>
+      <c r="D15" s="195" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -12136,36 +12124,36 @@
   <sheetData>
     <row r="1" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="D1" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="E1" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>130</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="33" t="s">
+        <v>131</v>
+      </c>
+      <c r="B2" s="33" t="s">
+        <v>132</v>
+      </c>
+      <c r="C2" s="33" t="s">
         <v>133</v>
-      </c>
-      <c r="B2" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="C2" s="33" t="s">
-        <v>135</v>
       </c>
       <c r="D2" s="33">
         <v>8</v>
@@ -12174,21 +12162,21 @@
         <v>2</v>
       </c>
       <c r="F2" s="33" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G2" s="34" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="33" t="s">
+        <v>136</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>137</v>
+      </c>
+      <c r="C3" s="33" t="s">
         <v>138</v>
-      </c>
-      <c r="B3" s="33" t="s">
-        <v>139</v>
-      </c>
-      <c r="C3" s="33" t="s">
-        <v>140</v>
       </c>
       <c r="D3" s="33">
         <v>5</v>
@@ -12197,10 +12185,10 @@
         <v>1</v>
       </c>
       <c r="F3" s="33" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G3" s="34" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -12393,24 +12381,24 @@
       <c r="G24" s="32"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="204" t="s">
-        <v>143</v>
-      </c>
-      <c r="B26" s="196"/>
-      <c r="C26" s="196"/>
-      <c r="D26" s="196"/>
-      <c r="E26" s="196"/>
-      <c r="F26" s="196"/>
-      <c r="G26" s="196"/>
+      <c r="A26" s="209" t="s">
+        <v>141</v>
+      </c>
+      <c r="B26" s="201"/>
+      <c r="C26" s="201"/>
+      <c r="D26" s="201"/>
+      <c r="E26" s="201"/>
+      <c r="F26" s="201"/>
+      <c r="G26" s="201"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="196"/>
-      <c r="B27" s="196"/>
-      <c r="C27" s="196"/>
-      <c r="D27" s="196"/>
-      <c r="E27" s="196"/>
-      <c r="F27" s="196"/>
-      <c r="G27" s="196"/>
+      <c r="A27" s="201"/>
+      <c r="B27" s="201"/>
+      <c r="C27" s="201"/>
+      <c r="D27" s="201"/>
+      <c r="E27" s="201"/>
+      <c r="F27" s="201"/>
+      <c r="G27" s="201"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>